<commit_message>
refactor(Télédéclarations): stocker la logique des champs simplifié/détaillé/obligatoires par année dans un fichier dédié (#7108)
</commit_message>
<xml_diff>
--- a/api/tests/files/diagnostics_complete/diagnostics_complete_good.xlsx
+++ b/api/tests/files/diagnostics_complete/diagnostics_complete_good.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -409,6 +409,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -468,8 +469,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -493,37 +498,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -599,884 +604,884 @@
   <dimension ref="A1:DU2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="48.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="25.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="47.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="19.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="41.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="23.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="45.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="19.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="42.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="17.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="40.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="15.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="37.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="31.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="33.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="31.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="26.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="30.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="26.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="24.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="22.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="34.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="36.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="35.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="29.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="33.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="30.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="28.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="26.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="25.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="27.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="25.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="20.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="0" width="23.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="0" width="20.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="0" width="18.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="0" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="0" width="33.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="0" width="35.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="0" width="34.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="0" width="28.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="0" width="32.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="0" width="29.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="0" width="27.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="0" width="25.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="0" width="24.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="55" min="55" style="0" width="26.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="56" min="56" style="0" width="25.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="57" min="57" style="0" width="19.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="58" style="0" width="23.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="59" min="59" style="0" width="20.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="60" min="60" style="0" width="18.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="61" min="61" style="0" width="15.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="62" min="62" style="0" width="38.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="63" min="63" style="0" width="40.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="0" width="39.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="0" width="33.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="0" width="37.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="0" width="34.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="0" width="32.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="0" width="30.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="0" width="27.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="0" width="29.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="0" width="28.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="0" width="22.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="0" width="26.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="75" min="75" style="0" width="23.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="76" min="76" style="0" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="77" min="77" style="0" width="18.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="78" min="78" style="0" width="31.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="79" style="0" width="33.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="80" min="80" style="0" width="32.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="81" min="81" style="0" width="26.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="82" min="82" style="0" width="30.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="83" min="83" style="0" width="26.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="84" min="84" style="0" width="24.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="85" min="85" style="0" width="22.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="86" min="86" style="0" width="32.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="87" min="87" style="0" width="34.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="88" min="88" style="0" width="32.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="89" min="89" style="0" width="27.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="90" min="90" style="0" width="31.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="91" min="91" style="0" width="27.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="92" min="92" style="0" width="25.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="93" min="93" style="0" width="23.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="94" min="94" style="0" width="31.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="95" min="95" style="0" width="33.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="96" min="96" style="0" width="31.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="97" min="97" style="0" width="26.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="98" min="98" style="0" width="30.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="99" min="99" style="0" width="26.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="100" min="100" style="0" width="24.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="101" min="101" style="0" width="22.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="102" style="0" width="27.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="103" min="103" style="0" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="104" min="104" style="0" width="27.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="105" min="105" style="0" width="22.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="106" min="106" style="0" width="26.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="107" min="107" style="0" width="22.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="108" min="108" style="0" width="20.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="109" min="109" style="0" width="18.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="110" min="110" style="0" width="32.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="111" min="111" style="0" width="33.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="112" min="112" style="0" width="32.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="113" min="113" style="0" width="27.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="114" min="114" style="0" width="30.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="115" min="115" style="0" width="27.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="116" min="116" style="0" width="25.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="117" min="117" style="0" width="23.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="118" min="118" style="0" width="25.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="119" min="119" style="0" width="27.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="120" min="120" style="0" width="26.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="121" min="121" style="0" width="21.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="122" min="122" style="0" width="24.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="123" min="123" style="0" width="21.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="124" min="124" style="0" width="19.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="125" min="125" style="0" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="46.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="26.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="48.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="25.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="47.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="19.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="41.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="23.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="45.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="42.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="17.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="40.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="15.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="37.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="33.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="31.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="26.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="30.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="26.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="24.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="22.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="34.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="36.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="35.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="29.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="33.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="30.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="28.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="25.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="27.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="25.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="20.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="23.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="20.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="18.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="33.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="35.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="34.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="28.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="1" width="32.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="1" width="29.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="1" width="27.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="1" width="25.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="1" width="24.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="55" min="55" style="1" width="26.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="56" min="56" style="1" width="25.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="57" min="57" style="1" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="58" style="1" width="23.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="59" min="59" style="1" width="20.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="60" min="60" style="1" width="18.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="61" min="61" style="1" width="15.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="62" min="62" style="1" width="38.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="63" min="63" style="1" width="40.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="39.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="33.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="37.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="34.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="32.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="30.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="27.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="28.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="22.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="26.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="75" min="75" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="76" min="76" style="1" width="21.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="77" min="77" style="1" width="18.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="78" min="78" style="1" width="31.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="79" style="1" width="33.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="80" min="80" style="1" width="32.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="81" min="81" style="1" width="26.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="82" min="82" style="1" width="30.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="83" min="83" style="1" width="26.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="84" min="84" style="1" width="24.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="85" min="85" style="1" width="22.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="86" min="86" style="1" width="32.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="87" min="87" style="1" width="34.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="88" min="88" style="1" width="32.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="89" min="89" style="1" width="27.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="90" min="90" style="1" width="31.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="91" min="91" style="1" width="27.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="92" min="92" style="1" width="25.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="93" min="93" style="1" width="23.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="94" min="94" style="1" width="31.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="95" min="95" style="1" width="33.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="96" min="96" style="1" width="31.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="97" min="97" style="1" width="26.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="98" min="98" style="1" width="30.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="99" min="99" style="1" width="26.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="100" min="100" style="1" width="24.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="101" min="101" style="1" width="22.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="102" style="1" width="27.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="103" min="103" style="1" width="29.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="104" min="104" style="1" width="27.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="105" min="105" style="1" width="22.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="106" min="106" style="1" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="107" min="107" style="1" width="22.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="108" min="108" style="1" width="20.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="109" min="109" style="1" width="18.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="110" min="110" style="1" width="32.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="111" min="111" style="1" width="33.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="112" min="112" style="1" width="32.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="113" min="113" style="1" width="27.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="114" min="114" style="1" width="30.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="115" min="115" style="1" width="27.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="116" min="116" style="1" width="25.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="117" min="117" style="1" width="23.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="118" min="118" style="1" width="25.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="119" min="119" style="1" width="27.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="120" min="120" style="1" width="26.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="121" min="121" style="1" width="21.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="122" min="122" style="1" width="24.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="123" min="123" style="1" width="21.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="124" min="124" style="1" width="19.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="125" min="125" style="1" width="17.15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="0" t="s">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="0" t="s">
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="0" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="0" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="0" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="0" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="0" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="0" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="0" t="s">
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="0" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="0" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="0" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="0" t="s">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="0" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="0" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="0" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="0" t="s">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="0" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="0" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="0" t="s">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="0" t="s">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="0" t="s">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="0" t="s">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="0" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="0" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="0" t="s">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="0" t="s">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="0" t="s">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="0" t="s">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="0" t="s">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="0" t="s">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="0" t="s">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="0" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="0" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="0" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="0" t="s">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="0" t="s">
+      <c r="BC1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="0" t="s">
+      <c r="BD1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="0" t="s">
+      <c r="BE1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" s="0" t="s">
+      <c r="BF1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" s="0" t="s">
+      <c r="BG1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="0" t="s">
+      <c r="BH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="0" t="s">
+      <c r="BI1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="0" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" s="0" t="s">
+      <c r="BK1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" s="0" t="s">
+      <c r="BL1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" s="0" t="s">
+      <c r="BM1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" s="0" t="s">
+      <c r="BN1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" s="0" t="s">
+      <c r="BO1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" s="0" t="s">
+      <c r="BP1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" s="0" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" s="0" t="s">
+      <c r="BR1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" s="0" t="s">
+      <c r="BS1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" s="0" t="s">
+      <c r="BT1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" s="0" t="s">
+      <c r="BU1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" s="0" t="s">
+      <c r="BV1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" s="0" t="s">
+      <c r="BW1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" s="0" t="s">
+      <c r="BX1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" s="0" t="s">
+      <c r="BY1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="BZ1" s="0" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="CA1" s="0" t="s">
+      <c r="CA1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="CB1" s="0" t="s">
+      <c r="CB1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="CC1" s="0" t="s">
+      <c r="CC1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="CD1" s="0" t="s">
+      <c r="CD1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="CE1" s="0" t="s">
+      <c r="CE1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="CF1" s="0" t="s">
+      <c r="CF1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" s="0" t="s">
+      <c r="CG1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" s="0" t="s">
+      <c r="CH1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" s="0" t="s">
+      <c r="CI1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" s="0" t="s">
+      <c r="CJ1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" s="0" t="s">
+      <c r="CK1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" s="0" t="s">
+      <c r="CL1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" s="0" t="s">
+      <c r="CM1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" s="0" t="s">
+      <c r="CN1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" s="0" t="s">
+      <c r="CO1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" s="0" t="s">
+      <c r="CP1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="CQ1" s="0" t="s">
+      <c r="CQ1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="CR1" s="0" t="s">
+      <c r="CR1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="CS1" s="0" t="s">
+      <c r="CS1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="CT1" s="0" t="s">
+      <c r="CT1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="CU1" s="0" t="s">
+      <c r="CU1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="CV1" s="0" t="s">
+      <c r="CV1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="CW1" s="0" t="s">
+      <c r="CW1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="CX1" s="0" t="s">
+      <c r="CX1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="CY1" s="0" t="s">
+      <c r="CY1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="CZ1" s="0" t="s">
+      <c r="CZ1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="DA1" s="0" t="s">
+      <c r="DA1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="DB1" s="0" t="s">
+      <c r="DB1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="DC1" s="0" t="s">
+      <c r="DC1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="DD1" s="0" t="s">
+      <c r="DD1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="DE1" s="0" t="s">
+      <c r="DE1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="DF1" s="0" t="s">
+      <c r="DF1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="DG1" s="0" t="s">
+      <c r="DG1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="DH1" s="0" t="s">
+      <c r="DH1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="DI1" s="0" t="s">
+      <c r="DI1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="DJ1" s="0" t="s">
+      <c r="DJ1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="DK1" s="0" t="s">
+      <c r="DK1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="DL1" s="0" t="s">
+      <c r="DL1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="DM1" s="0" t="s">
+      <c r="DM1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="DN1" s="0" t="s">
+      <c r="DN1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="DO1" s="0" t="s">
+      <c r="DO1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="DP1" s="0" t="s">
+      <c r="DP1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="DQ1" s="0" t="s">
+      <c r="DQ1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="DR1" s="0" t="s">
+      <c r="DR1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="DS1" s="0" t="s">
+      <c r="DS1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="DT1" s="0" t="s">
+      <c r="DT1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="DU1" s="0" t="s">
+      <c r="DU1" s="1" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>21340172201787</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C2" s="0" t="n">
+      <c r="B2" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="G2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="H2" s="0" t="n">
+      <c r="G2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="I2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="J2" s="0" t="n">
+      <c r="I2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="J2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="K2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="L2" s="0" t="n">
+      <c r="K2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="M2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="N2" s="0" t="n">
+      <c r="M2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="N2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="O2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="P2" s="0" t="n">
+      <c r="O2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="Q2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="R2" s="0" t="n">
+      <c r="Q2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="R2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="S2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="T2" s="0" t="n">
+      <c r="S2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="T2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="U2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="V2" s="0" t="n">
+      <c r="U2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="V2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="W2" s="0" t="n">
+      <c r="W2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="X2" s="0" t="n">
+      <c r="X2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="Y2" s="0" t="n">
+      <c r="Y2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="Z2" s="0" t="n">
+      <c r="Z2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="AA2" s="0" t="n">
+      <c r="AA2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="AB2" s="0" t="n">
+      <c r="AB2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="AC2" s="0" t="n">
+      <c r="AC2" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="AD2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AE2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AF2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AG2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AH2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AI2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AJ2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AK2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="AL2" s="0" t="n">
+      <c r="AD2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AE2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AF2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AG2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AH2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AI2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AJ2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AK2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AM2" s="0" t="n">
+      <c r="AM2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AN2" s="0" t="n">
+      <c r="AN2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AO2" s="0" t="n">
+      <c r="AO2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AP2" s="0" t="n">
+      <c r="AP2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AQ2" s="0" t="n">
+      <c r="AQ2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AR2" s="0" t="n">
+      <c r="AR2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AS2" s="0" t="n">
+      <c r="AS2" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="AT2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="AU2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="AV2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="AW2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="AX2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="AY2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="AZ2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BA2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BB2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BC2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BD2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BE2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BF2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BG2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BH2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BI2" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="BJ2" s="0" t="n">
+      <c r="AT2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="AU2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="AV2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="AW2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="AX2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="AY2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="AZ2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BA2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BB2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BC2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BD2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BE2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BF2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BG2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BH2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BI2" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="BJ2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BK2" s="0" t="n">
+      <c r="BK2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BL2" s="0" t="n">
+      <c r="BL2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BM2" s="0" t="n">
+      <c r="BM2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BN2" s="0" t="n">
+      <c r="BN2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BO2" s="0" t="n">
+      <c r="BO2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BP2" s="0" t="n">
+      <c r="BP2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BQ2" s="0" t="n">
+      <c r="BQ2" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="BR2" s="0" t="n">
+      <c r="BR2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BS2" s="0" t="n">
+      <c r="BS2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BT2" s="0" t="n">
+      <c r="BT2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BU2" s="0" t="n">
+      <c r="BU2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BV2" s="0" t="n">
+      <c r="BV2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BW2" s="0" t="n">
+      <c r="BW2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BX2" s="0" t="n">
+      <c r="BX2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BY2" s="0" t="n">
+      <c r="BY2" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="BZ2" s="0" t="n">
+      <c r="BZ2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CA2" s="0" t="n">
+      <c r="CA2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CB2" s="0" t="n">
+      <c r="CB2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CC2" s="0" t="n">
+      <c r="CC2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CD2" s="0" t="n">
+      <c r="CD2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CE2" s="0" t="n">
+      <c r="CE2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CF2" s="0" t="n">
+      <c r="CF2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CG2" s="0" t="n">
+      <c r="CG2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="CH2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CI2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CJ2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CK2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CL2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CM2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CN2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CO2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="CP2" s="0" t="n">
+      <c r="CH2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CI2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CJ2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CK2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CL2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CM2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CN2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CO2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CP2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CQ2" s="0" t="n">
+      <c r="CQ2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CR2" s="0" t="n">
+      <c r="CR2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CS2" s="0" t="n">
+      <c r="CS2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CT2" s="0" t="n">
+      <c r="CT2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CU2" s="0" t="n">
+      <c r="CU2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CV2" s="0" t="n">
+      <c r="CV2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CW2" s="0" t="n">
+      <c r="CW2" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="CX2" s="0" t="n">
+      <c r="CX2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="CY2" s="0" t="n">
+      <c r="CY2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="CZ2" s="0" t="n">
+      <c r="CZ2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="DA2" s="0" t="n">
+      <c r="DA2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="DB2" s="0" t="n">
+      <c r="DB2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="DC2" s="0" t="n">
+      <c r="DC2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="DD2" s="0" t="n">
+      <c r="DD2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="DE2" s="0" t="n">
+      <c r="DE2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="DF2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DG2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DH2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DI2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DJ2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DK2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DL2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DM2" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="DN2" s="0" t="n">
+      <c r="DF2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DG2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DH2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DI2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DJ2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DK2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DL2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DM2" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="DN2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DO2" s="0" t="n">
+      <c r="DO2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DP2" s="0" t="n">
+      <c r="DP2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DQ2" s="0" t="n">
+      <c r="DQ2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DR2" s="0" t="n">
+      <c r="DR2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DS2" s="0" t="n">
+      <c r="DS2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DT2" s="0" t="n">
+      <c r="DT2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="DU2" s="0" t="n">
+      <c r="DU2" s="1" t="n">
         <v>35</v>
       </c>
     </row>

</xml_diff>